<commit_message>
feat: shared bulk-import modals + user-bulk Excel templates
- MasterThesisBulkUploadModal: shared coordinator-side thesis import
  (preview → confirm), resolves academic year from Excel Batch column
- UsersBulkUploadModal: people-only bulk import for STUDENT/SUPERVISOR/EXTERNAL_EXAMINER
- New Excel templates: student_users_template.xlsx, supervisor_users_template.xlsx,
  external_users_template.xlsx (blank headers + sample rows)
- generate-samples.js extended to emit all user-bulk templates
- POST /users/bulk-import wired up in routes/users.js
</commit_message>
<xml_diff>
--- a/backend/excel-templates/master_upload_template.xlsx
+++ b/backend/excel-templates/master_upload_template.xlsx
@@ -462,7 +462,7 @@
         <v>Anup Baral</v>
       </c>
       <c r="B3" t="str">
-        <v>080MSCS001</v>
+        <v>080MSCS01</v>
       </c>
       <c r="C3" t="str">
         <v>Deep Learning for Nepali Sign Language Recognition</v>
@@ -491,7 +491,7 @@
         <v>Bina Thapa</v>
       </c>
       <c r="B4" t="str">
-        <v>080MSDSA001</v>
+        <v>080MSDSA01</v>
       </c>
       <c r="C4" t="str">
         <v>Predictive Analytics for Agricultural Yield in Nepal</v>

</xml_diff>